<commit_message>
BOEJ-4930: Update author / last updated by names in documents.
</commit_message>
<xml_diff>
--- a/GenBOE/RDM.Web/Templates/Export/RateCodesImportExample.xlsx
+++ b/GenBOE/RDM.Web/Templates/Export/RateCodesImportExample.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="19001"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brunworg\Source\Workspaces\genBOE\dev\GenBOE\RDM.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jueb\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{895319F2-96F8-4F43-84D0-54747DC3F0D4}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12510" windowHeight="6660"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rate Codes" sheetId="1" r:id="rId1"/>
@@ -114,8 +115,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -145,8 +146,36 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFECF0F1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFECF0F1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FF452DB2"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -156,6 +185,36 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor indexed="22"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF070729"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF9F9F9F"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF452DB2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD35714"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -182,9 +241,15 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -194,9 +259,15 @@
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="8">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
+    <cellStyle name="PPDuplicateRow" xfId="5" xr:uid="{2425B5C8-4471-4790-ACF0-609676229772}"/>
+    <cellStyle name="PPHeaderColumn" xfId="3" xr:uid="{EB6F58C2-5FF7-446A-B885-E647FDA8477E}"/>
+    <cellStyle name="PPHeaderRequired" xfId="4" xr:uid="{D2DF0C01-2205-4111-8D26-B6E33D1C2855}"/>
+    <cellStyle name="PPHeaderTop" xfId="2" xr:uid="{BF2C00F9-18DE-4627-A479-1F9605CB25B5}"/>
+    <cellStyle name="PPInvalidValue" xfId="6" xr:uid="{460EF8DA-0A36-426E-882E-7A3473954F42}"/>
+    <cellStyle name="PPMissingValue" xfId="7" xr:uid="{8B2E8A1F-A6FB-473F-A5D1-651EBB21C91D}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -507,7 +578,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:X1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -612,11 +683,19 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C_x000D__x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D__x000D_</oddFooter>
+    <evenHeader>&amp;C_x000D__x000D_</evenHeader>
+    <evenFooter>&amp;C_x000D__x000D_</evenFooter>
+    <firstHeader>&amp;C_x000D__x000D_</firstHeader>
+    <firstFooter>&amp;C_x000D__x000D_</firstFooter>
+  </headerFooter>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -651,5 +730,14 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <headerFooter>
+    <oddHeader>&amp;C_x000D__x000D_</oddHeader>
+    <oddFooter>&amp;C_x000D__x000D_</oddFooter>
+    <evenHeader>&amp;C_x000D__x000D_</evenHeader>
+    <evenFooter>&amp;C_x000D__x000D_</evenFooter>
+    <firstHeader>&amp;C_x000D__x000D_</firstHeader>
+    <firstFooter>&amp;C_x000D__x000D_</firstFooter>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated exporter code, Excel template
</commit_message>
<xml_diff>
--- a/GenBOE/RDM.Web/Templates/Export/RateCodesImportExample.xlsx
+++ b/GenBOE/RDM.Web/Templates/Export/RateCodesImportExample.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="22527"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jueb\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e309214\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{895319F2-96F8-4F43-84D0-54747DC3F0D4}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8827166C-CCFF-407D-8C9D-9A33A603F628}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="25440" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rate Codes" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="29">
   <si>
     <t>Rate Code</t>
   </si>
@@ -110,6 +110,18 @@
   </si>
   <si>
     <t>Description</t>
+  </si>
+  <si>
+    <t>ProPricer Description8</t>
+  </si>
+  <si>
+    <t>Resource Class8</t>
+  </si>
+  <si>
+    <t>ProPricer Description9</t>
+  </si>
+  <si>
+    <t>Resource Class9</t>
   </si>
 </sst>
 </file>
@@ -219,7 +231,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -240,6 +252,17 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -251,13 +274,16 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="8">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -579,7 +605,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:X1"/>
+  <dimension ref="A1:AB1"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.7109375" customWidth="1"/>
@@ -604,9 +630,10 @@
     <col min="22" max="22" width="15.140625" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="21.140625" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="25" max="28" width="21.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -673,10 +700,22 @@
       <c r="V1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="X1" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="Y1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="AA1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>

<commit_message>
PROPH-2207: Remove 1LMX Direct Labor Rates from RDM
</commit_message>
<xml_diff>
--- a/GenBOE/RDM.Web/Templates/Export/RateCodesImportExample.xlsx
+++ b/GenBOE/RDM.Web/Templates/Export/RateCodesImportExample.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\e403038\source\IES\GenBOE\RDM.Web\Templates\Export\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\gitBoe\GenBOE\RDM.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{776DA148-31F4-481C-B84F-C671DD68EE07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3934C99E-2477-4295-9354-7E4AA72E94C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15990" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22320" yWindow="30" windowWidth="34035" windowHeight="21570" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Rate Codes" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="30">
   <si>
     <t>Rate Code</t>
   </si>
@@ -126,276 +126,6 @@
   </si>
   <si>
     <t>Disclosure Type</t>
-  </si>
-  <si>
-    <t>ProPricer Description11</t>
-  </si>
-  <si>
-    <t>Resource Class11</t>
-  </si>
-  <si>
-    <t>ProPricer Description12</t>
-  </si>
-  <si>
-    <t>Resource Class12</t>
-  </si>
-  <si>
-    <t>ProPricer Description13</t>
-  </si>
-  <si>
-    <t>Resource Class13</t>
-  </si>
-  <si>
-    <t>ProPricer Description14</t>
-  </si>
-  <si>
-    <t>Resource Class14</t>
-  </si>
-  <si>
-    <t>ProPricer Description15</t>
-  </si>
-  <si>
-    <t>Resource Class15</t>
-  </si>
-  <si>
-    <t>ProPricer Description21</t>
-  </si>
-  <si>
-    <t>Resource Class21</t>
-  </si>
-  <si>
-    <t>ProPricer Description22</t>
-  </si>
-  <si>
-    <t>Resource Class22</t>
-  </si>
-  <si>
-    <t>ProPricer Description23</t>
-  </si>
-  <si>
-    <t>Resource Class23</t>
-  </si>
-  <si>
-    <t>ProPricer Description24</t>
-  </si>
-  <si>
-    <t>Resource Class24</t>
-  </si>
-  <si>
-    <t>ProPricer Description25</t>
-  </si>
-  <si>
-    <t>Resource Class25</t>
-  </si>
-  <si>
-    <t>ProPricer Description31</t>
-  </si>
-  <si>
-    <t>Resource Class31</t>
-  </si>
-  <si>
-    <t>ProPricer Description32</t>
-  </si>
-  <si>
-    <t>Resource Class32</t>
-  </si>
-  <si>
-    <t>ProPricer Description33</t>
-  </si>
-  <si>
-    <t>Resource Class33</t>
-  </si>
-  <si>
-    <t>ProPricer Description34</t>
-  </si>
-  <si>
-    <t>Resource Class34</t>
-  </si>
-  <si>
-    <t>ProPricer Description35</t>
-  </si>
-  <si>
-    <t>Resource Class35</t>
-  </si>
-  <si>
-    <t>ProPricer Description41</t>
-  </si>
-  <si>
-    <t>Resource Class41</t>
-  </si>
-  <si>
-    <t>ProPricer Description42</t>
-  </si>
-  <si>
-    <t>Resource Class42</t>
-  </si>
-  <si>
-    <t>ProPricer Description43</t>
-  </si>
-  <si>
-    <t>Resource Class43</t>
-  </si>
-  <si>
-    <t>ProPricer Description44</t>
-  </si>
-  <si>
-    <t>Resource Class44</t>
-  </si>
-  <si>
-    <t>ProPricer Description45</t>
-  </si>
-  <si>
-    <t>Resource Class45</t>
-  </si>
-  <si>
-    <t>ProPricer Description51</t>
-  </si>
-  <si>
-    <t>Resource Class51</t>
-  </si>
-  <si>
-    <t>ProPricer Description52</t>
-  </si>
-  <si>
-    <t>Resource Class52</t>
-  </si>
-  <si>
-    <t>ProPricer Description53</t>
-  </si>
-  <si>
-    <t>Resource Class53</t>
-  </si>
-  <si>
-    <t>ProPricer Description54</t>
-  </si>
-  <si>
-    <t>Resource Class54</t>
-  </si>
-  <si>
-    <t>ProPricer Description55</t>
-  </si>
-  <si>
-    <t>Resource Class55</t>
-  </si>
-  <si>
-    <t>ProPricer Description61</t>
-  </si>
-  <si>
-    <t>Resource Class61</t>
-  </si>
-  <si>
-    <t>ProPricer Description62</t>
-  </si>
-  <si>
-    <t>Resource Class62</t>
-  </si>
-  <si>
-    <t>ProPricer Description63</t>
-  </si>
-  <si>
-    <t>Resource Class63</t>
-  </si>
-  <si>
-    <t>ProPricer Description64</t>
-  </si>
-  <si>
-    <t>Resource Class64</t>
-  </si>
-  <si>
-    <t>ProPricer Description65</t>
-  </si>
-  <si>
-    <t>Resource Class65</t>
-  </si>
-  <si>
-    <t>ProPricer Description71</t>
-  </si>
-  <si>
-    <t>Resource Class71</t>
-  </si>
-  <si>
-    <t>ProPricer Description72</t>
-  </si>
-  <si>
-    <t>Resource Class72</t>
-  </si>
-  <si>
-    <t>ProPricer Description73</t>
-  </si>
-  <si>
-    <t>Resource Class73</t>
-  </si>
-  <si>
-    <t>ProPricer Description74</t>
-  </si>
-  <si>
-    <t>Resource Class74</t>
-  </si>
-  <si>
-    <t>ProPricer Description75</t>
-  </si>
-  <si>
-    <t>Resource Class75</t>
-  </si>
-  <si>
-    <t>ProPricer Description81</t>
-  </si>
-  <si>
-    <t>Resource Class81</t>
-  </si>
-  <si>
-    <t>ProPricer Description82</t>
-  </si>
-  <si>
-    <t>Resource Class82</t>
-  </si>
-  <si>
-    <t>ProPricer Description83</t>
-  </si>
-  <si>
-    <t>Resource Class83</t>
-  </si>
-  <si>
-    <t>ProPricer Description84</t>
-  </si>
-  <si>
-    <t>Resource Class84</t>
-  </si>
-  <si>
-    <t>ProPricer Description85</t>
-  </si>
-  <si>
-    <t>Resource Class85</t>
-  </si>
-  <si>
-    <t>ProPricer Description91</t>
-  </si>
-  <si>
-    <t>Resource Class91</t>
-  </si>
-  <si>
-    <t>ProPricer Description92</t>
-  </si>
-  <si>
-    <t>Resource Class92</t>
-  </si>
-  <si>
-    <t>ProPricer Description93</t>
-  </si>
-  <si>
-    <t>Resource Class93</t>
-  </si>
-  <si>
-    <t>ProPricer Description94</t>
-  </si>
-  <si>
-    <t>Resource Class94</t>
-  </si>
-  <si>
-    <t>ProPricer Description95</t>
-  </si>
-  <si>
-    <t>Resource Class95</t>
   </si>
 </sst>
 </file>
@@ -880,49 +610,40 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:DO1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AC1"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="7.7265625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.54296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.26953125" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="8.26953125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.26953125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.90625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="16.36328125" customWidth="1"/>
-    <col min="31" max="31" width="12.54296875" customWidth="1"/>
-    <col min="32" max="32" width="15.26953125" customWidth="1"/>
-    <col min="33" max="33" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="8.54296875" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="8.1796875" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="8.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="8.7109375" customWidth="1"/>
+    <col min="2" max="2" width="8.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" customWidth="1"/>
+    <col min="8" max="8" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="28" max="29" width="12.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:119" ht="31.5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:29" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -1005,279 +726,9 @@
         <v>28</v>
       </c>
       <c r="AB1" s="1" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="AC1" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="AD1" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="AE1" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AF1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="AG1" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="AH1" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="AI1" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="AJ1" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="AK1" s="4" t="s">
-        <v>39</v>
-      </c>
-      <c r="AL1" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AM1" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="AN1" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="AO1" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="AP1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="AQ1" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="AR1" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="AS1" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="AT1" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="AU1" s="4" t="s">
-        <v>49</v>
-      </c>
-      <c r="AV1" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="AW1" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="AX1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="AY1" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="AZ1" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="BA1" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="BB1" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="BC1" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="BD1" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="BE1" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="BF1" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="BG1" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="BH1" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="BI1" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="BJ1" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="BK1" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="BL1" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="BM1" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="BN1" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="BO1" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="BP1" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="BQ1" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="BR1" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="BS1" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="BT1" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="BU1" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="BV1" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="BW1" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="BX1" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="BY1" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="BZ1" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="CA1" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="CB1" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="CC1" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="CD1" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="CE1" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="CF1" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="CG1" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="CH1" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="CI1" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="CJ1" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="CK1" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="CL1" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="CM1" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="CN1" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="CO1" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="CP1" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="CQ1" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="CR1" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="CS1" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="CT1" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="CU1" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="CV1" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="CW1" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="CX1" s="1" t="s">
-        <v>104</v>
-      </c>
-      <c r="CY1" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="CZ1" s="4" t="s">
-        <v>106</v>
-      </c>
-      <c r="DA1" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="DB1" s="4" t="s">
-        <v>108</v>
-      </c>
-      <c r="DC1" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="DD1" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="DE1" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="DF1" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="DG1" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="DH1" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="DI1" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="DJ1" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="DK1" s="4" t="s">
-        <v>117</v>
-      </c>
-      <c r="DL1" s="4" t="s">
-        <v>118</v>
-      </c>
-      <c r="DM1" s="4" t="s">
-        <v>119</v>
-      </c>
-      <c r="DN1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="DO1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -1298,16 +749,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="30.7265625" style="3" customWidth="1"/>
+    <col min="1" max="2" width="30.7109375" style="3" customWidth="1"/>
     <col min="3" max="3" width="14" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.26953125" style="3" customWidth="1"/>
-    <col min="5" max="6" width="18.26953125" style="3" customWidth="1"/>
-    <col min="7" max="7" width="18.453125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="13.28515625" style="3" customWidth="1"/>
+    <col min="5" max="6" width="18.28515625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="18.42578125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>2</v>
       </c>

</xml_diff>

<commit_message>
PROPH-2207: Hiding a column that is no longer necessary
</commit_message>
<xml_diff>
--- a/GenBOE/RDM.Web/Templates/Export/RateCodesImportExample.xlsx
+++ b/GenBOE/RDM.Web/Templates/Export/RateCodesImportExample.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\gitBoe\GenBOE\RDM.Web\Templates\Export\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3934C99E-2477-4295-9354-7E4AA72E94C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7336CD25-8AB7-4C9A-AE0F-2BEF3DB56AAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22320" yWindow="30" windowWidth="34035" windowHeight="21570" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -619,7 +619,7 @@
     <col min="4" max="4" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="12.28515625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.28515625" customWidth="1"/>
+    <col min="7" max="7" width="14.28515625" hidden="1" customWidth="1"/>
     <col min="8" max="8" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18.140625" bestFit="1" customWidth="1"/>

</xml_diff>